<commit_message>
collect_results: count beads with molecule_counts
Bead counts now come from the same function as the simulation, so gel
fraction and volume shrinkage also work for spaced molecules. This also
corrects job 03f1d195 (12.5 %), whose job document says 1250
tetrathiols; the recipe and its first frame show the simulation had 625.
Results and plots regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/analysis/results/results.xlsx
+++ b/analysis/results/results.xlsx
@@ -650,7 +650,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Spacer setting (0 = simple 4-bead ene monomer)</t>
+          <t>Spacer beads between the two C=C of the di-ene (0 = E=E-E=E)</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Spacer setting (0 = simple 2-bead dithiol)</t>
+          <t>Spacer beads between the two SH of the dithiol (0 = S-S)</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Total beads in the box (simple molecules only)</t>
+          <t>Total beads in the box (without the 4 placeholder beads)</t>
         </is>
       </c>
     </row>
@@ -1141,9 +1141,9 @@
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="19" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="21" customWidth="1" min="22" max="22"/>
     <col width="27" customWidth="1" min="23" max="23"/>
@@ -2422,22 +2422,22 @@
         <v>5</v>
       </c>
       <c r="O5" t="n">
-        <v>750</v>
+        <v>625</v>
       </c>
       <c r="P5" t="n">
-        <v>279.5084971874737</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>8500</v>
+        <v>8750</v>
       </c>
       <c r="R5" t="n">
-        <v>559.0169943749473</v>
+        <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>60750</v>
+        <v>60625</v>
       </c>
       <c r="T5" t="n">
-        <v>279.5084971874742</v>
+        <v>0</v>
       </c>
       <c r="U5" t="n">
         <v>1840100</v>
@@ -2470,10 +2470,10 @@
         <v>0.006041189607639224</v>
       </c>
       <c r="AE5" t="n">
-        <v>7.612630968230585</v>
+        <v>7.423540123711334</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.3832577962487003</v>
+        <v>0.07076732074060622</v>
       </c>
       <c r="AG5" t="n">
         <v>0.9387495881182648</v>
@@ -2500,10 +2500,10 @@
         <v>61.67090075554272</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.6595290553334736</v>
+        <v>0.6608626804123711</v>
       </c>
       <c r="AP5" t="n">
-        <v>0.07327763967394603</v>
+        <v>0.07304856606203743</v>
       </c>
       <c r="AQ5" t="n">
         <v>1399.4</v>
@@ -14283,13 +14283,13 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>1250</v>
+        <v>625</v>
       </c>
       <c r="Q39" t="n">
-        <v>7500</v>
+        <v>8750</v>
       </c>
       <c r="R39" t="n">
-        <v>61250</v>
+        <v>60625</v>
       </c>
       <c r="S39" t="n">
         <v>1729100</v>
@@ -14307,7 +14307,7 @@
         <v>0.9607925139840033</v>
       </c>
       <c r="X39" t="n">
-        <v>8.29094040816326</v>
+        <v>7.345486185567007</v>
       </c>
       <c r="Y39" t="n">
         <v>0.9406168322007318</v>
@@ -14322,7 +14322,7 @@
         <v>1261</v>
       </c>
       <c r="AC39" t="n">
-        <v>0.6468081632653061</v>
+        <v>0.6534762886597938</v>
       </c>
       <c r="AD39" t="n">
         <v>1410</v>

</xml_diff>